<commit_message>
enhance inventory management UI with action cards and modals
</commit_message>
<xml_diff>
--- a/tests/fixtures/inventarios/inventario_arka_pruebas.xlsx
+++ b/tests/fixtures/inventarios/inventario_arka_pruebas.xlsx
@@ -4,7 +4,11 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Inventario" sheetId="1" r:id="rId1"/>
+    <sheet name="Casos de prueba" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Inventario!$A$1:$N$29</definedName>
+  </definedNames>
 </workbook>
 </file>
 
@@ -397,20 +401,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L21"/>
+  <dimension ref="A1:N29"/>
   <cols>
-    <col min="1" max="1" width="18.83203125" customWidth="1"/>
-    <col min="2" max="2" width="18.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="18.83203125" customWidth="1"/>
-    <col min="5" max="5" width="18.83203125" customWidth="1"/>
-    <col min="6" max="6" width="18.83203125" customWidth="1"/>
-    <col min="7" max="7" width="18.83203125" customWidth="1"/>
-    <col min="8" max="8" width="18.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="1" max="1" width="16.83203125" customWidth="1"/>
+    <col min="2" max="2" width="16.83203125" customWidth="1"/>
+    <col min="3" max="3" width="16.83203125" customWidth="1"/>
+    <col min="4" max="4" width="16.83203125" customWidth="1"/>
+    <col min="5" max="5" width="16.83203125" customWidth="1"/>
+    <col min="6" max="6" width="16.83203125" customWidth="1"/>
+    <col min="7" max="7" width="16.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="16.83203125" customWidth="1"/>
     <col min="10" max="10" width="18.83203125" customWidth="1"/>
-    <col min="11" max="11" width="18.83203125" customWidth="1"/>
-    <col min="12" max="12" width="18.83203125" customWidth="1"/>
+    <col min="11" max="11" width="16.83203125" customWidth="1"/>
+    <col min="12" max="12" width="16.83203125" customWidth="1"/>
+    <col min="13" max="13" width="16.83203125" customWidth="1"/>
+    <col min="14" max="14" width="21.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -450,770 +456,1617 @@
       <c r="L1" t="str">
         <v>PLACA LOCAL</v>
       </c>
+      <c r="M1" t="str">
+        <v>ETIQUETADO</v>
+      </c>
+      <c r="N1" t="str">
+        <v>NOMBRE DEL MATERIAL</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>QA-ARKA-001-7171</v>
+        <v>ARKA-TEST-001</v>
       </c>
       <c r="B2" t="str">
-        <v>Equipo QA Medidor digital de pH 1</v>
+        <v>Microscopio óptico compuesto</v>
       </c>
       <c r="C2" t="str">
-        <v>Marca de prueba Uno</v>
+        <v>Marca Demo</v>
       </c>
       <c r="D2" t="str">
-        <v>MODELO-QA-001-6174</v>
+        <v>M-100</v>
       </c>
       <c r="E2" t="str">
-        <v>SERIE-QA-001-3269</v>
+        <v>SER-EQP-001</v>
       </c>
       <c r="F2" t="str">
-        <v>Proveedor ficticio QA-1</v>
+        <v>Proveedor Genérico</v>
       </c>
       <c r="G2" t="str">
-        <v>Dato sintético de prueba; no corresponde a inventario real.</v>
+        <v>Caso válido con datos opcionales.</v>
       </c>
       <c r="H2" t="str">
-        <v>CODIGO-QA-001-2851</v>
+        <v>INT-EQP-001</v>
       </c>
       <c r="I2" t="str">
-        <v>ID-QA-001-8820</v>
+        <v>ID-EQP-001</v>
       </c>
       <c r="J2" t="str">
-        <v>BARRAS-QA-001-1627</v>
+        <v>BAR-EQP-001</v>
       </c>
       <c r="K2" t="str">
-        <v>QR-QA-001-4951</v>
+        <v>QR-EQP-001</v>
       </c>
       <c r="L2" t="str">
-        <v>LOCAL-QA-001-7686</v>
+        <v>LOC-EQP-001</v>
+      </c>
+      <c r="M2" t="str">
+        <v>TAG-EQP-001</v>
+      </c>
+      <c r="N2" t="str">
+        <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>QA-ARKA-002-1445</v>
+        <v>ARKA-TEST-002</v>
       </c>
       <c r="B3" t="str">
-        <v>Equipo QA Centrífuga de mesa 2</v>
+        <v>Balanza analítica</v>
       </c>
       <c r="C3" t="str">
-        <v>Marca QA Sur</v>
+        <v/>
       </c>
       <c r="D3" t="str">
-        <v>MODELO-QA-002-5639</v>
+        <v/>
       </c>
       <c r="E3" t="str">
-        <v>SERIE-QA-002-4720</v>
+        <v/>
       </c>
       <c r="F3" t="str">
-        <v>Proveedor ficticio QA-1</v>
+        <v/>
       </c>
       <c r="G3" t="str">
-        <v>Dato sintético de prueba; no corresponde a inventario real.</v>
+        <v/>
       </c>
       <c r="H3" t="str">
-        <v>CODIGO-QA-002-4933</v>
+        <v/>
       </c>
       <c r="I3" t="str">
-        <v>ID-QA-002-2145</v>
+        <v/>
       </c>
       <c r="J3" t="str">
-        <v>BARRAS-QA-002-1594</v>
+        <v/>
       </c>
       <c r="K3" t="str">
-        <v>QR-QA-002-1036</v>
+        <v/>
       </c>
       <c r="L3" t="str">
-        <v>LOCAL-QA-002-4252</v>
+        <v/>
+      </c>
+      <c r="M3" t="str">
+        <v/>
+      </c>
+      <c r="N3" t="str">
+        <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>QA-ARKA-003-2444</v>
+        <v>ARKA-TEST-003</v>
       </c>
       <c r="B4" t="str">
-        <v>Equipo QA Cabina de flujo laminar 3</v>
+        <v>Agitador magnético</v>
       </c>
       <c r="C4" t="str">
-        <v>Marca QA Centro</v>
+        <v>Genérica</v>
       </c>
       <c r="D4" t="str">
-        <v>MODELO-QA-003-3797</v>
+        <v>AG-20</v>
       </c>
       <c r="E4" t="str">
-        <v>SERIE-QA-003-4877</v>
+        <v>SER-EQP-003</v>
       </c>
       <c r="F4" t="str">
-        <v>Proveedor ficticio QA-1</v>
+        <v/>
       </c>
       <c r="G4" t="str">
-        <v>Dato sintético de prueba; no corresponde a inventario real.</v>
+        <v/>
       </c>
       <c r="H4" t="str">
-        <v>CODIGO-QA-003-4914</v>
+        <v/>
       </c>
       <c r="I4" t="str">
-        <v>ID-QA-003-3973</v>
+        <v/>
       </c>
       <c r="J4" t="str">
-        <v>BARRAS-QA-003-6407</v>
+        <v/>
       </c>
       <c r="K4" t="str">
-        <v>QR-QA-003-2662</v>
+        <v/>
       </c>
       <c r="L4" t="str">
-        <v>LOCAL-QA-003-7442</v>
+        <v/>
+      </c>
+      <c r="M4" t="str">
+        <v/>
+      </c>
+      <c r="N4" t="str">
+        <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>QA-ARKA-004-1589</v>
+        <v/>
       </c>
       <c r="B5" t="str">
-        <v>Equipo QA Microscopio binocular 4</v>
+        <v>Microscopio estereoscópico</v>
       </c>
       <c r="C5" t="str">
-        <v>Marca QA Sur</v>
+        <v/>
       </c>
       <c r="D5" t="str">
-        <v>MODELO-QA-004-2168</v>
+        <v/>
       </c>
       <c r="E5" t="str">
-        <v>SERIE-QA-004-4585</v>
+        <v/>
       </c>
       <c r="F5" t="str">
-        <v>Proveedor ficticio QA-2</v>
+        <v/>
       </c>
       <c r="G5" t="str">
-        <v>Dato sintético de prueba; no corresponde a inventario real.</v>
+        <v/>
       </c>
       <c r="H5" t="str">
-        <v>CODIGO-QA-004-9952</v>
+        <v/>
       </c>
       <c r="I5" t="str">
-        <v>ID-QA-004-6336</v>
+        <v/>
       </c>
       <c r="J5" t="str">
-        <v>BARRAS-QA-004-3981</v>
+        <v/>
       </c>
       <c r="K5" t="str">
-        <v>QR-QA-004-8889</v>
+        <v/>
       </c>
       <c r="L5" t="str">
-        <v>LOCAL-QA-004-5405</v>
+        <v/>
+      </c>
+      <c r="M5" t="str">
+        <v/>
+      </c>
+      <c r="N5" t="str">
+        <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>QA-ARKA-005-7874</v>
+        <v>ARKA-TEST-005</v>
       </c>
       <c r="B6" t="str">
-        <v>Equipo QA Fuente de alimentación 5</v>
+        <v/>
       </c>
       <c r="C6" t="str">
-        <v>Marca QA Centro</v>
+        <v/>
       </c>
       <c r="D6" t="str">
-        <v>MODELO-QA-005-7286</v>
+        <v/>
       </c>
       <c r="E6" t="str">
-        <v>SERIE-QA-005-2126</v>
+        <v/>
       </c>
       <c r="F6" t="str">
-        <v>Proveedor ficticio QA-2</v>
+        <v/>
       </c>
       <c r="G6" t="str">
-        <v>Dato sintético de prueba; no corresponde a inventario real.</v>
+        <v/>
       </c>
       <c r="H6" t="str">
-        <v>CODIGO-QA-005-9800</v>
+        <v/>
       </c>
       <c r="I6" t="str">
-        <v>ID-QA-005-2137</v>
+        <v/>
       </c>
       <c r="J6" t="str">
-        <v>BARRAS-QA-005-4655</v>
+        <v/>
       </c>
       <c r="K6" t="str">
-        <v>QR-QA-005-2445</v>
+        <v/>
       </c>
       <c r="L6" t="str">
-        <v>LOCAL-QA-005-6442</v>
+        <v/>
+      </c>
+      <c r="M6" t="str">
+        <v/>
+      </c>
+      <c r="N6" t="str">
+        <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>QA-ARKA-006-4353</v>
+        <v>arka-test-001</v>
       </c>
       <c r="B7" t="str">
-        <v>Equipo QA Pipeta de volumen variable 6</v>
+        <v>Equipo con placa repetida</v>
       </c>
       <c r="C7" t="str">
-        <v>Marca QA Sur</v>
+        <v/>
       </c>
       <c r="D7" t="str">
-        <v>MODELO-QA-006-2875</v>
+        <v/>
       </c>
       <c r="E7" t="str">
-        <v>SERIE-QA-006-7502</v>
+        <v/>
       </c>
       <c r="F7" t="str">
-        <v>Proveedor de pruebas</v>
+        <v/>
       </c>
       <c r="G7" t="str">
-        <v>Dato sintético de prueba; no corresponde a inventario real.</v>
+        <v/>
       </c>
       <c r="H7" t="str">
-        <v>CODIGO-QA-006-1523</v>
+        <v/>
       </c>
       <c r="I7" t="str">
-        <v>ID-QA-006-7714</v>
+        <v/>
       </c>
       <c r="J7" t="str">
-        <v>BARRAS-QA-006-1302</v>
+        <v/>
       </c>
       <c r="K7" t="str">
-        <v>QR-QA-006-6172</v>
+        <v/>
       </c>
       <c r="L7" t="str">
-        <v>LOCAL-QA-006-4319</v>
+        <v/>
+      </c>
+      <c r="M7" t="str">
+        <v/>
+      </c>
+      <c r="N7" t="str">
+        <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>QA-ARKA-007-4743</v>
+        <v>ARKA-TEST-007</v>
       </c>
       <c r="B8" t="str">
-        <v>Equipo QA Estufa de secado 7</v>
+        <v>Equipo con QR repetido</v>
       </c>
       <c r="C8" t="str">
-        <v>Marca de prueba Uno</v>
+        <v/>
       </c>
       <c r="D8" t="str">
-        <v>MODELO-QA-007-9177</v>
+        <v/>
       </c>
       <c r="E8" t="str">
-        <v>SERIE-QA-007-7926</v>
+        <v/>
       </c>
       <c r="F8" t="str">
-        <v>Proveedor de pruebas</v>
+        <v/>
       </c>
       <c r="G8" t="str">
-        <v>Dato sintético de prueba; no corresponde a inventario real.</v>
+        <v/>
       </c>
       <c r="H8" t="str">
-        <v>CODIGO-QA-007-3432</v>
+        <v/>
       </c>
       <c r="I8" t="str">
-        <v>ID-QA-007-4587</v>
+        <v/>
       </c>
       <c r="J8" t="str">
-        <v>BARRAS-QA-007-6190</v>
+        <v/>
       </c>
       <c r="K8" t="str">
-        <v>QR-QA-007-3426</v>
+        <v>QR-EQP-001</v>
       </c>
       <c r="L8" t="str">
-        <v>LOCAL-QA-007-7904</v>
+        <v/>
+      </c>
+      <c r="M8" t="str">
+        <v/>
+      </c>
+      <c r="N8" t="str">
+        <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>QA-ARKA-008-1226</v>
+        <v>PPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPPP</v>
       </c>
       <c r="B9" t="str">
-        <v>Equipo QA Medidor digital de pH 8</v>
+        <v>Equipo con placa demasiado larga</v>
       </c>
       <c r="C9" t="str">
-        <v>Marca QA Sur</v>
+        <v/>
       </c>
       <c r="D9" t="str">
-        <v>MODELO-QA-008-2672</v>
+        <v/>
       </c>
       <c r="E9" t="str">
-        <v>SERIE-QA-008-4825</v>
+        <v/>
       </c>
       <c r="F9" t="str">
-        <v>Proveedor ficticio QA-1</v>
+        <v/>
       </c>
       <c r="G9" t="str">
-        <v>Dato sintético de prueba; no corresponde a inventario real.</v>
+        <v/>
       </c>
       <c r="H9" t="str">
-        <v>CODIGO-QA-008-7145</v>
+        <v/>
       </c>
       <c r="I9" t="str">
-        <v>ID-QA-008-2803</v>
+        <v/>
       </c>
       <c r="J9" t="str">
-        <v>BARRAS-QA-008-3932</v>
+        <v/>
       </c>
       <c r="K9" t="str">
-        <v>QR-QA-008-1131</v>
+        <v/>
       </c>
       <c r="L9" t="str">
-        <v>LOCAL-QA-008-6187</v>
+        <v/>
+      </c>
+      <c r="M9" t="str">
+        <v/>
+      </c>
+      <c r="N9" t="str">
+        <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>QA-ARKA-009-6305</v>
+        <v>ARKA-TEST-009</v>
       </c>
       <c r="B10" t="str">
-        <v>Equipo QA Agitador magnético 9</v>
+        <v>Equipo con serie demasiado larga</v>
       </c>
       <c r="C10" t="str">
-        <v>Marca QA Sur</v>
+        <v/>
       </c>
       <c r="D10" t="str">
-        <v>MODELO-QA-009-2553</v>
+        <v/>
       </c>
       <c r="E10" t="str">
-        <v>SERIE-QA-009-5916</v>
+        <v>SSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSSS</v>
       </c>
       <c r="F10" t="str">
-        <v>Proveedor de pruebas</v>
+        <v/>
       </c>
       <c r="G10" t="str">
-        <v>Dato sintético de prueba; no corresponde a inventario real.</v>
+        <v/>
       </c>
       <c r="H10" t="str">
-        <v>CODIGO-QA-009-7339</v>
+        <v/>
       </c>
       <c r="I10" t="str">
-        <v>ID-QA-009-6211</v>
+        <v/>
       </c>
       <c r="J10" t="str">
-        <v>BARRAS-QA-009-2175</v>
+        <v/>
       </c>
       <c r="K10" t="str">
-        <v>QR-QA-009-5668</v>
+        <v/>
       </c>
       <c r="L10" t="str">
-        <v>LOCAL-QA-009-4231</v>
+        <v/>
+      </c>
+      <c r="M10" t="str">
+        <v/>
+      </c>
+      <c r="N10" t="str">
+        <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>QA-ARKA-010-2004</v>
+        <v>ARKA-TEST-010</v>
       </c>
       <c r="B11" t="str">
-        <v>Equipo QA Estufa de secado 10</v>
+        <v>DDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDDD</v>
       </c>
       <c r="C11" t="str">
-        <v>Marca QA Sur</v>
+        <v/>
       </c>
       <c r="D11" t="str">
-        <v>MODELO-QA-010-5289</v>
+        <v/>
       </c>
       <c r="E11" t="str">
-        <v>SERIE-QA-010-1845</v>
+        <v/>
       </c>
       <c r="F11" t="str">
-        <v>Proveedor de pruebas</v>
+        <v/>
       </c>
       <c r="G11" t="str">
-        <v>Dato sintético de prueba; no corresponde a inventario real.</v>
+        <v/>
       </c>
       <c r="H11" t="str">
-        <v>CODIGO-QA-010-2041</v>
+        <v/>
       </c>
       <c r="I11" t="str">
-        <v>ID-QA-010-1879</v>
+        <v/>
       </c>
       <c r="J11" t="str">
-        <v>BARRAS-QA-010-9736</v>
+        <v/>
       </c>
       <c r="K11" t="str">
-        <v>QR-QA-010-1618</v>
+        <v/>
       </c>
       <c r="L11" t="str">
-        <v>LOCAL-QA-010-6029</v>
+        <v/>
+      </c>
+      <c r="M11" t="str">
+        <v/>
+      </c>
+      <c r="N11" t="str">
+        <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>QA-ARKA-011-5197</v>
+        <v>ARKA-TEST-011</v>
       </c>
       <c r="B12" t="str">
-        <v>Equipo QA Estufa de secado 11</v>
+        <v>Equipo con observación extensa</v>
       </c>
       <c r="C12" t="str">
-        <v>Marca QA Norte</v>
+        <v/>
       </c>
       <c r="D12" t="str">
-        <v>MODELO-QA-011-1584</v>
+        <v/>
       </c>
       <c r="E12" t="str">
-        <v>SERIE-QA-011-8973</v>
+        <v/>
       </c>
       <c r="F12" t="str">
-        <v>Proveedor ficticio QA-2</v>
+        <v/>
       </c>
       <c r="G12" t="str">
-        <v>Dato sintético de prueba; no corresponde a inventario real.</v>
+        <v>OOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOOO</v>
       </c>
       <c r="H12" t="str">
-        <v>CODIGO-QA-011-8082</v>
+        <v/>
       </c>
       <c r="I12" t="str">
-        <v>ID-QA-011-8308</v>
+        <v/>
       </c>
       <c r="J12" t="str">
-        <v>BARRAS-QA-011-3404</v>
+        <v/>
       </c>
       <c r="K12" t="str">
-        <v>QR-QA-011-6473</v>
+        <v/>
       </c>
       <c r="L12" t="str">
-        <v>LOCAL-QA-011-1037</v>
+        <v/>
+      </c>
+      <c r="M12" t="str">
+        <v/>
+      </c>
+      <c r="N12" t="str">
+        <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>QA-ARKA-012-2191</v>
+        <v>ARKA-TEST-012</v>
       </c>
       <c r="B13" t="str">
-        <v>Equipo QA Baño termostatado 12</v>
+        <v>Microscopio</v>
       </c>
       <c r="C13" t="str">
-        <v>Marca QA Centro</v>
+        <v/>
       </c>
       <c r="D13" t="str">
-        <v>MODELO-QA-012-2561</v>
+        <v/>
       </c>
       <c r="E13" t="str">
-        <v>SERIE-QA-012-2971</v>
+        <v/>
       </c>
       <c r="F13" t="str">
-        <v>Proveedor ficticio QA-1</v>
+        <v/>
       </c>
       <c r="G13" t="str">
-        <v>Dato sintético de prueba; no corresponde a inventario real.</v>
+        <v/>
       </c>
       <c r="H13" t="str">
-        <v>CODIGO-QA-012-8132</v>
+        <v/>
       </c>
       <c r="I13" t="str">
-        <v>ID-QA-012-6110</v>
+        <v/>
       </c>
       <c r="J13" t="str">
-        <v>BARRAS-QA-012-6747</v>
+        <v/>
       </c>
       <c r="K13" t="str">
-        <v>QR-QA-012-8272</v>
+        <v/>
       </c>
       <c r="L13" t="str">
-        <v>LOCAL-QA-012-6170</v>
+        <v/>
+      </c>
+      <c r="M13" t="str">
+        <v/>
+      </c>
+      <c r="N13" t="str">
+        <v>Balanza</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>QA-ARKA-013-7140</v>
+        <v>ARKA-TEST-013</v>
       </c>
       <c r="B14" t="str">
-        <v>Equipo QA Fuente de alimentación 13</v>
+        <v>Equipo con identificador extenso</v>
       </c>
       <c r="C14" t="str">
-        <v>Marca QA Sur</v>
+        <v/>
       </c>
       <c r="D14" t="str">
-        <v>MODELO-QA-013-1528</v>
+        <v/>
       </c>
       <c r="E14" t="str">
-        <v>SERIE-QA-013-2931</v>
+        <v/>
       </c>
       <c r="F14" t="str">
-        <v>Proveedor ficticio QA-1</v>
+        <v/>
       </c>
       <c r="G14" t="str">
-        <v>Dato sintético de prueba; no corresponde a inventario real.</v>
+        <v/>
       </c>
       <c r="H14" t="str">
-        <v>CODIGO-QA-013-9311</v>
+        <v/>
       </c>
       <c r="I14" t="str">
-        <v>ID-QA-013-9760</v>
+        <v>IIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIIII</v>
       </c>
       <c r="J14" t="str">
-        <v>BARRAS-QA-013-8629</v>
+        <v/>
       </c>
       <c r="K14" t="str">
-        <v>QR-QA-013-8508</v>
+        <v/>
       </c>
       <c r="L14" t="str">
-        <v>LOCAL-QA-013-3088</v>
+        <v/>
+      </c>
+      <c r="M14" t="str">
+        <v/>
+      </c>
+      <c r="N14" t="str">
+        <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>QA-ARKA-014-3953</v>
+        <v>ARKA-ADIC-001</v>
       </c>
       <c r="B15" t="str">
-        <v>Equipo QA Cabina de flujo laminar 14</v>
+        <v>Equipo de laboratorio de prueba 001</v>
       </c>
       <c r="C15" t="str">
-        <v>Marca QA Norte</v>
+        <v>Marca Demo</v>
       </c>
       <c r="D15" t="str">
-        <v>MODELO-QA-014-5408</v>
+        <v>MD-001</v>
       </c>
       <c r="E15" t="str">
-        <v>SERIE-QA-014-1278</v>
+        <v>SER-ADIC-001</v>
       </c>
       <c r="F15" t="str">
-        <v>Proveedor ficticio QA-2</v>
+        <v>Proveedor Genérico</v>
       </c>
       <c r="G15" t="str">
-        <v>Dato sintético de prueba; no corresponde a inventario real.</v>
+        <v>Caso exitoso adicional 001.</v>
       </c>
       <c r="H15" t="str">
-        <v>CODIGO-QA-014-6566</v>
+        <v>INT-EQP-ADIC-001</v>
       </c>
       <c r="I15" t="str">
-        <v>ID-QA-014-2391</v>
+        <v>ID-EQP-ADIC-001</v>
       </c>
       <c r="J15" t="str">
-        <v>BARRAS-QA-014-2954</v>
+        <v>BAR-EQP-ADIC-001</v>
       </c>
       <c r="K15" t="str">
-        <v>QR-QA-014-3386</v>
+        <v>QR-EQP-ADIC-001</v>
       </c>
       <c r="L15" t="str">
-        <v>LOCAL-QA-014-6027</v>
+        <v>LOC-EQP-ADIC-001</v>
+      </c>
+      <c r="M15" t="str">
+        <v>TAG-EQP-ADIC-001</v>
+      </c>
+      <c r="N15" t="str">
+        <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>QA-ARKA-015-6169</v>
+        <v>ARKA-ADIC-002</v>
       </c>
       <c r="B16" t="str">
-        <v>Equipo QA Agitador magnético 15</v>
+        <v>Equipo de laboratorio de prueba 002</v>
       </c>
       <c r="C16" t="str">
-        <v>Marca QA Centro</v>
+        <v>Marca Demo</v>
       </c>
       <c r="D16" t="str">
-        <v>MODELO-QA-015-4140</v>
+        <v>MD-002</v>
       </c>
       <c r="E16" t="str">
-        <v>SERIE-QA-015-9731</v>
+        <v>SER-ADIC-002</v>
       </c>
       <c r="F16" t="str">
-        <v>Proveedor ficticio QA-2</v>
+        <v>Proveedor Genérico</v>
       </c>
       <c r="G16" t="str">
-        <v>Dato sintético de prueba; no corresponde a inventario real.</v>
+        <v>Caso exitoso adicional 002.</v>
       </c>
       <c r="H16" t="str">
-        <v>CODIGO-QA-015-8503</v>
+        <v>INT-EQP-ADIC-002</v>
       </c>
       <c r="I16" t="str">
-        <v>ID-QA-015-4591</v>
+        <v>ID-EQP-ADIC-002</v>
       </c>
       <c r="J16" t="str">
-        <v>BARRAS-QA-015-4738</v>
+        <v>BAR-EQP-ADIC-002</v>
       </c>
       <c r="K16" t="str">
-        <v>QR-QA-015-4910</v>
+        <v>QR-EQP-ADIC-002</v>
       </c>
       <c r="L16" t="str">
-        <v>LOCAL-QA-015-4515</v>
+        <v>LOC-EQP-ADIC-002</v>
+      </c>
+      <c r="M16" t="str">
+        <v>TAG-EQP-ADIC-002</v>
+      </c>
+      <c r="N16" t="str">
+        <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>QA-ARKA-016-4621</v>
+        <v>ARKA-ADIC-003</v>
       </c>
       <c r="B17" t="str">
-        <v>Equipo QA Centrífuga de mesa 16</v>
+        <v>Equipo de laboratorio de prueba 003</v>
       </c>
       <c r="C17" t="str">
-        <v>Marca de prueba Uno</v>
+        <v>Marca Demo</v>
       </c>
       <c r="D17" t="str">
-        <v>MODELO-QA-016-6415</v>
+        <v>MD-003</v>
       </c>
       <c r="E17" t="str">
-        <v>SERIE-QA-016-2222</v>
+        <v>SER-ADIC-003</v>
       </c>
       <c r="F17" t="str">
-        <v>Proveedor ficticio QA-2</v>
+        <v>Proveedor Genérico</v>
       </c>
       <c r="G17" t="str">
-        <v>Dato sintético de prueba; no corresponde a inventario real.</v>
+        <v>Caso exitoso adicional 003.</v>
       </c>
       <c r="H17" t="str">
-        <v>CODIGO-QA-016-5377</v>
+        <v>INT-EQP-ADIC-003</v>
       </c>
       <c r="I17" t="str">
-        <v>ID-QA-016-5435</v>
+        <v>ID-EQP-ADIC-003</v>
       </c>
       <c r="J17" t="str">
-        <v>BARRAS-QA-016-5695</v>
+        <v>BAR-EQP-ADIC-003</v>
       </c>
       <c r="K17" t="str">
-        <v>QR-QA-016-5574</v>
+        <v>QR-EQP-ADIC-003</v>
       </c>
       <c r="L17" t="str">
-        <v>LOCAL-QA-016-4322</v>
+        <v>LOC-EQP-ADIC-003</v>
+      </c>
+      <c r="M17" t="str">
+        <v>TAG-EQP-ADIC-003</v>
+      </c>
+      <c r="N17" t="str">
+        <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>QA-ARKA-017-5566</v>
+        <v>ARKA-ADIC-004</v>
       </c>
       <c r="B18" t="str">
-        <v>Equipo QA Baño termostatado 17</v>
+        <v>Equipo de laboratorio de prueba 004</v>
       </c>
       <c r="C18" t="str">
-        <v>Marca QA Norte</v>
+        <v>Marca Demo</v>
       </c>
       <c r="D18" t="str">
-        <v>MODELO-QA-017-4853</v>
+        <v>MD-004</v>
       </c>
       <c r="E18" t="str">
-        <v>SERIE-QA-017-6288</v>
+        <v>SER-ADIC-004</v>
       </c>
       <c r="F18" t="str">
-        <v>Proveedor ficticio QA-1</v>
+        <v>Proveedor Genérico</v>
       </c>
       <c r="G18" t="str">
-        <v>Dato sintético de prueba; no corresponde a inventario real.</v>
+        <v>Caso exitoso adicional 004.</v>
       </c>
       <c r="H18" t="str">
-        <v>CODIGO-QA-017-8149</v>
+        <v>INT-EQP-ADIC-004</v>
       </c>
       <c r="I18" t="str">
-        <v>ID-QA-017-8425</v>
+        <v>ID-EQP-ADIC-004</v>
       </c>
       <c r="J18" t="str">
-        <v>BARRAS-QA-017-4555</v>
+        <v>BAR-EQP-ADIC-004</v>
       </c>
       <c r="K18" t="str">
-        <v>QR-QA-017-4019</v>
+        <v>QR-EQP-ADIC-004</v>
       </c>
       <c r="L18" t="str">
-        <v>LOCAL-QA-017-1889</v>
+        <v>LOC-EQP-ADIC-004</v>
+      </c>
+      <c r="M18" t="str">
+        <v>TAG-EQP-ADIC-004</v>
+      </c>
+      <c r="N18" t="str">
+        <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>QA-ARKA-018-2442</v>
+        <v>ARKA-ADIC-005</v>
       </c>
       <c r="B19" t="str">
-        <v>Equipo QA Medidor digital de pH 18</v>
+        <v>Equipo de laboratorio de prueba 005</v>
       </c>
       <c r="C19" t="str">
-        <v>Marca QA Norte</v>
+        <v>Marca Demo</v>
       </c>
       <c r="D19" t="str">
-        <v>MODELO-QA-018-1296</v>
+        <v>MD-005</v>
       </c>
       <c r="E19" t="str">
-        <v>SERIE-QA-018-4272</v>
+        <v>SER-ADIC-005</v>
       </c>
       <c r="F19" t="str">
-        <v>Proveedor ficticio QA-2</v>
+        <v>Proveedor Genérico</v>
       </c>
       <c r="G19" t="str">
-        <v>Dato sintético de prueba; no corresponde a inventario real.</v>
+        <v>Caso exitoso adicional 005.</v>
       </c>
       <c r="H19" t="str">
-        <v>CODIGO-QA-018-5319</v>
+        <v>INT-EQP-ADIC-005</v>
       </c>
       <c r="I19" t="str">
-        <v>ID-QA-018-8234</v>
+        <v>ID-EQP-ADIC-005</v>
       </c>
       <c r="J19" t="str">
-        <v>BARRAS-QA-018-4623</v>
+        <v>BAR-EQP-ADIC-005</v>
       </c>
       <c r="K19" t="str">
-        <v>QR-QA-018-4222</v>
+        <v>QR-EQP-ADIC-005</v>
       </c>
       <c r="L19" t="str">
-        <v>LOCAL-QA-018-6540</v>
+        <v>LOC-EQP-ADIC-005</v>
+      </c>
+      <c r="M19" t="str">
+        <v>TAG-EQP-ADIC-005</v>
+      </c>
+      <c r="N19" t="str">
+        <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>QA-ARKA-019-4730</v>
+        <v>ARKA-ADIC-006</v>
       </c>
       <c r="B20" t="str">
-        <v>Equipo QA Pipeta de volumen variable 19</v>
+        <v>Equipo de laboratorio de prueba 006</v>
       </c>
       <c r="C20" t="str">
-        <v>Marca QA Centro</v>
+        <v>Marca Demo</v>
       </c>
       <c r="D20" t="str">
-        <v>MODELO-QA-019-2466</v>
+        <v>MD-006</v>
       </c>
       <c r="E20" t="str">
-        <v>SERIE-QA-019-5136</v>
+        <v>SER-ADIC-006</v>
       </c>
       <c r="F20" t="str">
-        <v>Proveedor ficticio QA-1</v>
+        <v>Proveedor Genérico</v>
       </c>
       <c r="G20" t="str">
-        <v>Dato sintético de prueba; no corresponde a inventario real.</v>
+        <v>Caso exitoso adicional 006.</v>
       </c>
       <c r="H20" t="str">
-        <v>CODIGO-QA-019-4383</v>
+        <v>INT-EQP-ADIC-006</v>
       </c>
       <c r="I20" t="str">
-        <v>ID-QA-019-2718</v>
+        <v>ID-EQP-ADIC-006</v>
       </c>
       <c r="J20" t="str">
-        <v>BARRAS-QA-019-6872</v>
+        <v>BAR-EQP-ADIC-006</v>
       </c>
       <c r="K20" t="str">
-        <v>QR-QA-019-4337</v>
+        <v>QR-EQP-ADIC-006</v>
       </c>
       <c r="L20" t="str">
-        <v>LOCAL-QA-019-9431</v>
+        <v>LOC-EQP-ADIC-006</v>
+      </c>
+      <c r="M20" t="str">
+        <v>TAG-EQP-ADIC-006</v>
+      </c>
+      <c r="N20" t="str">
+        <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>QA-ARKA-020-7095</v>
+        <v>ARKA-ADIC-007</v>
       </c>
       <c r="B21" t="str">
-        <v>Equipo QA Balanza de precisión 20</v>
+        <v>Equipo de laboratorio de prueba 007</v>
       </c>
       <c r="C21" t="str">
-        <v>Marca QA Centro</v>
+        <v>Marca Demo</v>
       </c>
       <c r="D21" t="str">
-        <v>MODELO-QA-020-3722</v>
+        <v>MD-007</v>
       </c>
       <c r="E21" t="str">
-        <v>SERIE-QA-020-2480</v>
+        <v>SER-ADIC-007</v>
       </c>
       <c r="F21" t="str">
-        <v>Proveedor de pruebas</v>
+        <v>Proveedor Genérico</v>
       </c>
       <c r="G21" t="str">
-        <v>Dato sintético de prueba; no corresponde a inventario real.</v>
+        <v>Caso exitoso adicional 007.</v>
       </c>
       <c r="H21" t="str">
-        <v>CODIGO-QA-020-5902</v>
+        <v>INT-EQP-ADIC-007</v>
       </c>
       <c r="I21" t="str">
-        <v>ID-QA-020-7409</v>
+        <v>ID-EQP-ADIC-007</v>
       </c>
       <c r="J21" t="str">
-        <v>BARRAS-QA-020-8593</v>
+        <v>BAR-EQP-ADIC-007</v>
       </c>
       <c r="K21" t="str">
-        <v>QR-QA-020-7364</v>
+        <v>QR-EQP-ADIC-007</v>
       </c>
       <c r="L21" t="str">
-        <v>LOCAL-QA-020-4972</v>
+        <v>LOC-EQP-ADIC-007</v>
+      </c>
+      <c r="M21" t="str">
+        <v>TAG-EQP-ADIC-007</v>
+      </c>
+      <c r="N21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>ARKA-ADIC-008</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Equipo de laboratorio de prueba 008</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Marca Demo</v>
+      </c>
+      <c r="D22" t="str">
+        <v>MD-008</v>
+      </c>
+      <c r="E22" t="str">
+        <v>SER-ADIC-008</v>
+      </c>
+      <c r="F22" t="str">
+        <v>Proveedor Genérico</v>
+      </c>
+      <c r="G22" t="str">
+        <v>Caso exitoso adicional 008.</v>
+      </c>
+      <c r="H22" t="str">
+        <v>INT-EQP-ADIC-008</v>
+      </c>
+      <c r="I22" t="str">
+        <v>ID-EQP-ADIC-008</v>
+      </c>
+      <c r="J22" t="str">
+        <v>BAR-EQP-ADIC-008</v>
+      </c>
+      <c r="K22" t="str">
+        <v>QR-EQP-ADIC-008</v>
+      </c>
+      <c r="L22" t="str">
+        <v>LOC-EQP-ADIC-008</v>
+      </c>
+      <c r="M22" t="str">
+        <v>TAG-EQP-ADIC-008</v>
+      </c>
+      <c r="N22" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>ARKA-ADIC-009</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Equipo de laboratorio de prueba 009</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Marca Demo</v>
+      </c>
+      <c r="D23" t="str">
+        <v>MD-009</v>
+      </c>
+      <c r="E23" t="str">
+        <v>SER-ADIC-009</v>
+      </c>
+      <c r="F23" t="str">
+        <v>Proveedor Genérico</v>
+      </c>
+      <c r="G23" t="str">
+        <v>Caso exitoso adicional 009.</v>
+      </c>
+      <c r="H23" t="str">
+        <v>INT-EQP-ADIC-009</v>
+      </c>
+      <c r="I23" t="str">
+        <v>ID-EQP-ADIC-009</v>
+      </c>
+      <c r="J23" t="str">
+        <v>BAR-EQP-ADIC-009</v>
+      </c>
+      <c r="K23" t="str">
+        <v>QR-EQP-ADIC-009</v>
+      </c>
+      <c r="L23" t="str">
+        <v>LOC-EQP-ADIC-009</v>
+      </c>
+      <c r="M23" t="str">
+        <v>TAG-EQP-ADIC-009</v>
+      </c>
+      <c r="N23" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>ARKA-ADIC-010</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Equipo de laboratorio de prueba 010</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Marca Demo</v>
+      </c>
+      <c r="D24" t="str">
+        <v>MD-010</v>
+      </c>
+      <c r="E24" t="str">
+        <v>SER-ADIC-010</v>
+      </c>
+      <c r="F24" t="str">
+        <v>Proveedor Genérico</v>
+      </c>
+      <c r="G24" t="str">
+        <v>Caso exitoso adicional 010.</v>
+      </c>
+      <c r="H24" t="str">
+        <v>INT-EQP-ADIC-010</v>
+      </c>
+      <c r="I24" t="str">
+        <v>ID-EQP-ADIC-010</v>
+      </c>
+      <c r="J24" t="str">
+        <v>BAR-EQP-ADIC-010</v>
+      </c>
+      <c r="K24" t="str">
+        <v>QR-EQP-ADIC-010</v>
+      </c>
+      <c r="L24" t="str">
+        <v>LOC-EQP-ADIC-010</v>
+      </c>
+      <c r="M24" t="str">
+        <v>TAG-EQP-ADIC-010</v>
+      </c>
+      <c r="N24" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>ARKA-ADIC-011</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Equipo de laboratorio de prueba 011</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Marca Demo</v>
+      </c>
+      <c r="D25" t="str">
+        <v>MD-011</v>
+      </c>
+      <c r="E25" t="str">
+        <v>SER-ADIC-011</v>
+      </c>
+      <c r="F25" t="str">
+        <v>Proveedor Genérico</v>
+      </c>
+      <c r="G25" t="str">
+        <v>Caso exitoso adicional 011.</v>
+      </c>
+      <c r="H25" t="str">
+        <v>INT-EQP-ADIC-011</v>
+      </c>
+      <c r="I25" t="str">
+        <v>ID-EQP-ADIC-011</v>
+      </c>
+      <c r="J25" t="str">
+        <v>BAR-EQP-ADIC-011</v>
+      </c>
+      <c r="K25" t="str">
+        <v>QR-EQP-ADIC-011</v>
+      </c>
+      <c r="L25" t="str">
+        <v>LOC-EQP-ADIC-011</v>
+      </c>
+      <c r="M25" t="str">
+        <v>TAG-EQP-ADIC-011</v>
+      </c>
+      <c r="N25" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>ARKA-ADIC-012</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Equipo de laboratorio de prueba 012</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Marca Demo</v>
+      </c>
+      <c r="D26" t="str">
+        <v>MD-012</v>
+      </c>
+      <c r="E26" t="str">
+        <v>SER-ADIC-012</v>
+      </c>
+      <c r="F26" t="str">
+        <v>Proveedor Genérico</v>
+      </c>
+      <c r="G26" t="str">
+        <v>Caso exitoso adicional 012.</v>
+      </c>
+      <c r="H26" t="str">
+        <v>INT-EQP-ADIC-012</v>
+      </c>
+      <c r="I26" t="str">
+        <v>ID-EQP-ADIC-012</v>
+      </c>
+      <c r="J26" t="str">
+        <v>BAR-EQP-ADIC-012</v>
+      </c>
+      <c r="K26" t="str">
+        <v>QR-EQP-ADIC-012</v>
+      </c>
+      <c r="L26" t="str">
+        <v>LOC-EQP-ADIC-012</v>
+      </c>
+      <c r="M26" t="str">
+        <v>TAG-EQP-ADIC-012</v>
+      </c>
+      <c r="N26" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>ARKA-ADIC-013</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Equipo de laboratorio de prueba 013</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Marca Demo</v>
+      </c>
+      <c r="D27" t="str">
+        <v>MD-013</v>
+      </c>
+      <c r="E27" t="str">
+        <v>SER-ADIC-013</v>
+      </c>
+      <c r="F27" t="str">
+        <v>Proveedor Genérico</v>
+      </c>
+      <c r="G27" t="str">
+        <v>Caso exitoso adicional 013.</v>
+      </c>
+      <c r="H27" t="str">
+        <v>INT-EQP-ADIC-013</v>
+      </c>
+      <c r="I27" t="str">
+        <v>ID-EQP-ADIC-013</v>
+      </c>
+      <c r="J27" t="str">
+        <v>BAR-EQP-ADIC-013</v>
+      </c>
+      <c r="K27" t="str">
+        <v>QR-EQP-ADIC-013</v>
+      </c>
+      <c r="L27" t="str">
+        <v>LOC-EQP-ADIC-013</v>
+      </c>
+      <c r="M27" t="str">
+        <v>TAG-EQP-ADIC-013</v>
+      </c>
+      <c r="N27" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>ARKA-ADIC-014</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Equipo de laboratorio de prueba 014</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Marca Demo</v>
+      </c>
+      <c r="D28" t="str">
+        <v>MD-014</v>
+      </c>
+      <c r="E28" t="str">
+        <v>SER-ADIC-014</v>
+      </c>
+      <c r="F28" t="str">
+        <v>Proveedor Genérico</v>
+      </c>
+      <c r="G28" t="str">
+        <v>Caso exitoso adicional 014.</v>
+      </c>
+      <c r="H28" t="str">
+        <v>INT-EQP-ADIC-014</v>
+      </c>
+      <c r="I28" t="str">
+        <v>ID-EQP-ADIC-014</v>
+      </c>
+      <c r="J28" t="str">
+        <v>BAR-EQP-ADIC-014</v>
+      </c>
+      <c r="K28" t="str">
+        <v>QR-EQP-ADIC-014</v>
+      </c>
+      <c r="L28" t="str">
+        <v>LOC-EQP-ADIC-014</v>
+      </c>
+      <c r="M28" t="str">
+        <v>TAG-EQP-ADIC-014</v>
+      </c>
+      <c r="N28" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>ARKA-ADIC-015</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Equipo de laboratorio de prueba 015</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Marca Demo</v>
+      </c>
+      <c r="D29" t="str">
+        <v>MD-015</v>
+      </c>
+      <c r="E29" t="str">
+        <v>SER-ADIC-015</v>
+      </c>
+      <c r="F29" t="str">
+        <v>Proveedor Genérico</v>
+      </c>
+      <c r="G29" t="str">
+        <v>Caso exitoso adicional 015.</v>
+      </c>
+      <c r="H29" t="str">
+        <v>INT-EQP-ADIC-015</v>
+      </c>
+      <c r="I29" t="str">
+        <v>ID-EQP-ADIC-015</v>
+      </c>
+      <c r="J29" t="str">
+        <v>BAR-EQP-ADIC-015</v>
+      </c>
+      <c r="K29" t="str">
+        <v>QR-EQP-ADIC-015</v>
+      </c>
+      <c r="L29" t="str">
+        <v>LOC-EQP-ADIC-015</v>
+      </c>
+      <c r="M29" t="str">
+        <v>TAG-EQP-ADIC-015</v>
+      </c>
+      <c r="N29" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:N29"/>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:N29"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C32"/>
+  <cols>
+    <col min="1" max="1" width="20.83203125" customWidth="1"/>
+    <col min="2" max="2" width="22.83203125" customWidth="1"/>
+    <col min="3" max="3" width="78.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Fila en Inventario</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Resultado esperado</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Caso de prueba</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>2</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Exitosa</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Registro completo con identificadores opcionales.</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>3</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Exitosa</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Registro válido mínimo con los campos obligatorios.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>4</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Exitosa</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Equipo válido con marca, modelo y serie.</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>5</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Fallida</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Error intencional: falta la placa oficial.</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>6</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Fallida</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Error intencional: falta la descripción.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>7</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Fallida</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Error intencional: placa duplicada (no distingue mayúsculas/minúsculas).</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>8</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Fallida</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Error intencional: código QR ya usado en otra fila.</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>9</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Fallida</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Error intencional: placa de más de 50 caracteres.</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>10</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Fallida</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Error intencional: serie de más de 100 caracteres.</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>11</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Fallida</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Error intencional: descripción de más de 1000 caracteres.</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>12</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Fallida</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Error intencional: observaciones de más de 2000 caracteres.</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>13</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Fallida</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Error intencional: DESCRIPCIÓN y NOMBRE DEL MATERIAL se contradicen.</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>14</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Fallida</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Error intencional: identificador ID de más de 255 caracteres.</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15">
+        <v>15</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Exitosa</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Registro válido adicional 001.</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16">
+        <v>16</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Exitosa</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Registro válido adicional 002.</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17">
+        <v>17</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Exitosa</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Registro válido adicional 003.</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18">
+        <v>18</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Exitosa</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Registro válido adicional 004.</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19">
+        <v>19</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Exitosa</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Registro válido adicional 005.</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20">
+        <v>20</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Exitosa</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Registro válido adicional 006.</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21">
+        <v>21</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Exitosa</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Registro válido adicional 007.</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22">
+        <v>22</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Exitosa</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Registro válido adicional 008.</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23">
+        <v>23</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Exitosa</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Registro válido adicional 009.</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24">
+        <v>24</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Exitosa</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Registro válido adicional 010.</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25">
+        <v>25</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Exitosa</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Registro válido adicional 011.</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26">
+        <v>26</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Exitosa</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Registro válido adicional 012.</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27">
+        <v>27</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Exitosa</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Registro válido adicional 013.</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28">
+        <v>28</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Exitosa</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Registro válido adicional 014.</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29">
+        <v>29</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Exitosa</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Registro válido adicional 015.</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v/>
+      </c>
+      <c r="B30" t="str">
+        <v/>
+      </c>
+      <c r="C30" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>Uso</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Carga únicamente la hoja Inventario; esta hoja documenta los resultados esperados.</v>
+      </c>
+      <c r="C31" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>Nota</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Los casos fallidos son intencionales y sirven para verificar las validaciones del cargue.</v>
+      </c>
+      <c r="C32" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C32"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>